<commit_message>
feat(buqi): adopt infinite ten-slot run baseline
</commit_message>
<xml_diff>
--- a/Design/Excel/GameHot/Datas/Buqi/BuqiGlobal.xlsx
+++ b/Design/Excel/GameHot/Datas/Buqi/BuqiGlobal.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BuqiGlobal" sheetId="1" r:id="Rf2aadb15f05c4fc7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BuqiGlobal" sheetId="1" r:id="R9a295a8d39c947eb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -356,7 +356,7 @@
         <x:v>content version</x:v>
       </x:c>
       <x:c r="D2" t="str">
-        <x:v>buqi-content-cv2</x:v>
+        <x:v>buqi-content-cv3</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -426,7 +426,7 @@
         <x:v>board slots</x:v>
       </x:c>
       <x:c r="D7" t="n">
-        <x:v>8</x:v>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="8">

</xml_diff>